<commit_message>
add lesson 1.8 bootstrap CI in excel and python
</commit_message>
<xml_diff>
--- a/lesson-1-8-bootstrap/bakery_bootstrap.xlsx
+++ b/lesson-1-8-bootstrap/bakery_bootstrap.xlsx
@@ -17,10 +17,9 @@
     <sheet name="Bootstrap" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlchart.v1.0" hidden="1">Bootstrap!$K$2:$K$1002</definedName>
+    <definedName name="_xlchart.v1.0" hidden="1">Bootstrap!$L$2:$L$1002</definedName>
     <definedName name="_xlchart.v1.1" hidden="1">Bootstrap!$L$2:$L$1002</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">Bootstrap!$L$2:$L$1002</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">Bootstrap!$K$2:$K$1002</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">Bootstrap!$K$2:$K$1002</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
@@ -810,7 +809,7 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.3</cx:f>
+        <cx:f>_xlchart.v1.2</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -899,7 +898,7 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.1</cx:f>
+        <cx:f>_xlchart.v1.0</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>

</xml_diff>